<commit_message>
docs: make submission checks self-contained
</commit_message>
<xml_diff>
--- a/docs/shtab-tasks-submission.xlsx
+++ b/docs/shtab-tasks-submission.xlsx
@@ -401,7 +401,7 @@
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="48.83203125" customWidth="1"/>
-    <col min="3" max="3" width="110.83203125" customWidth="1"/>
+    <col min="3" max="3" width="140.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -412,7 +412,7 @@
         <v>Ссылка</v>
       </c>
       <c r="C1" t="str">
-        <v>Инструкция</v>
+        <v>Самодостаточная инструкция для проверки</v>
       </c>
     </row>
     <row r="2">
@@ -423,7 +423,7 @@
         <v>http://111.88.245.141</v>
       </c>
       <c r="C2" t="str">
-        <v>Открыть лендинг. Проверить описание продукта: инструмент для штаба кампании, где главный технолог ведёт задачи из голоса, файлов, календаря и канбана.</v>
+        <v>Откройте http://111.88.245.141. На главной странице показан продукт «Штабные задачи»: веб-приложение и Telegram-бот для главного технолога избирательной кампании. Проверьте, что лендинг объясняет прикладную задачу: фиксировать поручения штаба, вести ответственных, дедлайны, календарь, канбан, голосовые задачи и задачи из протоколов встреч. Ожидаемый результат: по странице понятно, какую реальную задачу решает сервис и для кого он сделан.</v>
       </c>
     </row>
     <row r="3">
@@ -434,7 +434,7 @@
         <v>https://github.com/antiqueee/shtabtasks/commits/main</v>
       </c>
       <c r="C3" t="str">
-        <v>Открыть историю коммитов. Проект собран итеративно AI-агентами Claude/Codex по фазам: скелет, бот, календарь, протоколы, RAG, дашборд, деплой.</v>
+        <v>Откройте ссылку на историю коммитов GitHub. В истории видны последовательные AI-итерации проекта: скелет приложения, база данных, Telegram-бот, календарь, протоколы, RAG-ассистент, дашборд, деплой и исправления после проверки. Проект был собран в формате вайб-кодинга с Claude/Codex: разработка велась фазами через промпты, после фаз выполнялись коммиты и деплой. Ожидаемый результат: история репозитория подтверждает итеративную AI-разработку, а не один ручной монолитный коммит.</v>
       </c>
     </row>
     <row r="4">
@@ -445,7 +445,7 @@
         <v>http://111.88.245.141/app/protocols</v>
       </c>
       <c r="C4" t="str">
-        <v>Войти, открыть скрытую страницу протоколов, вставить текст протокола с поручениями и нажать Разобрать протокол. Задачи создаются через LLM-парсинг.</v>
+        <v>Откройте ссылку. Если появится экран входа, войдите: логин toniem2@mail.ru, пароль X7mP2vK9qL4bZ1rW. На странице «Протоколы и файлы» вставьте в поле текста пример: Протокол встречи. Ивану подготовить список агитаторов до пятницы 18:00. Марии проверить макеты листовок завтра. Петру собрать отчёт по дворам. Нажмите «Разобрать протокол». Ожидаемый результат: LLM извлечёт поручения из свободного текста и создаст отдельные задачи в системе.</v>
       </c>
     </row>
     <row r="5">
@@ -456,7 +456,7 @@
         <v>https://t.me/zadachishtaba2026_bot</v>
       </c>
       <c r="C5" t="str">
-        <v>Открыть бота, отправить текст или голосовое сообщение с задачей. Проверить появление задачи в веб-интерфейсе.</v>
+        <v>Откройте Telegram-бота @zadachishtaba2026_bot и нажмите Start. Отправьте текст: Завтра в 17:00 подготовить отчёт по агитации, ответственный Иван, тег агитация. Затем откройте веб-интерфейс http://111.88.245.141/app/board и войдите: toniem2@mail.ru / X7mP2vK9qL4bZ1rW. Ожидаемый результат: задача из Telegram появляется на канбан-доске в колонке «К выполнению» с названием, дедлайном, ответственным и тегом.</v>
       </c>
     </row>
     <row r="6">
@@ -467,7 +467,7 @@
         <v>http://111.88.245.141</v>
       </c>
       <c r="C6" t="str">
-        <v>Открыть публичную главную страницу без авторизации. На ней есть описание продукта, сценарии работы, фичи и кнопка входа.</v>
+        <v>Откройте http://111.88.245.141 без авторизации. Проверьте наличие публичной страницы продукта: заголовок про календарь задач штаба, описание сценария использования, блок «Как это работает», блок возможностей и кнопку «Войти». Ожидаемый результат: лендинг доступен без логина и объясняет продукт до входа в приложение.</v>
       </c>
     </row>
     <row r="7">
@@ -478,7 +478,7 @@
         <v>http://111.88.245.141/app/board</v>
       </c>
       <c r="C7" t="str">
-        <v>Войти и открыть канбан. Проверить создание, редактирование, перемещение и удаление задач.</v>
+        <v>Откройте ссылку. Если появится login, войдите: toniem2@mail.ru / X7mP2vK9qL4bZ1rW. На канбан-доске создайте задачу через верхнюю форму, например: название Проверить штабной список, ответственный Иван, тег Оргработа, дата/время на завтра. Затем откройте созданную задачу/редактирование, измените текст, переместите её между колонками или удалите. Ожидаемый результат: веб-страница работает как основной User Interface для управления задачами.</v>
       </c>
     </row>
     <row r="8">
@@ -489,7 +489,7 @@
         <v>http://111.88.245.141/login</v>
       </c>
       <c r="C8" t="str">
-        <v>Открыть страницу входа, войти: toniem2@mail.ru / X7mP2vK9qL4bZ1rW. Без входа рабочие страницы недоступны.</v>
+        <v>Откройте http://111.88.245.141/app/board в приватном окне браузера. Ожидаемый результат: вместо доски произойдёт редирект на страницу входа. На странице входа введите логин toniem2@mail.ru и пароль X7mP2vK9qL4bZ1rW, нажмите вход. Ожидаемый результат: после успешной авторизации открываются защищённые страницы приложения.</v>
       </c>
     </row>
     <row r="9">
@@ -500,7 +500,7 @@
         <v>http://111.88.245.141/app/assistant</v>
       </c>
       <c r="C9" t="str">
-        <v>Сначала загрузить протокол на /app/protocols, затем открыть ассистента и задать вопрос по содержимому протокола. Ответ строится по сохранённым фрагментам.</v>
+        <v>Сначала откройте http://111.88.245.141/app/protocols и войдите: toniem2@mail.ru / X7mP2vK9qL4bZ1rW. Вставьте текст протокола: На встрече решили: Иван отвечает за агитаторов, Мария за макеты листовок, Пётр за отчёт по дворам. Нажмите «Разобрать протокол». Затем откройте http://111.88.245.141/app/assistant и задайте вопрос: Кто отвечает за макеты листовок? Ожидаемый результат: ассистент отвечает на основе загруженного протокола и показывает источник/фрагмент.</v>
       </c>
     </row>
     <row r="10">
@@ -511,7 +511,7 @@
         <v>https://github.com/antiqueee/shtabtasks/blob/main/packages/db/src/schema.ts</v>
       </c>
       <c r="C10" t="str">
-        <v>Открыть схему Drizzle/Postgres. Есть таблицы пользователей, задач, ответственных, тегов, протоколов, чанков RAG, импортов и событий.</v>
+        <v>Откройте ссылку на файл схемы базы данных в репозитории. Проверьте, что проект использует Postgres через Drizzle ORM: в схеме описаны таблицы пользователей, задач, ответственных, тегов, шаблонов регулярных задач, протоколов, чанков протоколов для RAG, импортов и связей задач с импортами. Ожидаемый результат: наличие полноценной базы данных подтверждается схемой и связями сущностей.</v>
       </c>
     </row>
     <row r="11">
@@ -522,7 +522,7 @@
         <v>https://t.me/zadachishtaba2026_bot</v>
       </c>
       <c r="C11" t="str">
-        <v>Отправить голосовое сообщение в бот. Бот распознаёт речь через Speech-to-Text и создаёт задачу.</v>
+        <v>Откройте Telegram-бота @zadachishtaba2026_bot и отправьте голосовое сообщение, например произнесите: завтра в 12 подготовить отчёт по наблюдателям, ответственный Иван. Затем откройте http://111.88.245.141/app/board и войдите: toniem2@mail.ru / X7mP2vK9qL4bZ1rW. Ожидаемый результат: бот распознаёт голос через speech-to-text, превращает его в текст задачи и создаёт задачу на доске.</v>
       </c>
     </row>
     <row r="12">
@@ -533,7 +533,7 @@
         <v>http://111.88.245.141/app/dashboard</v>
       </c>
       <c r="C12" t="str">
-        <v>Войти и открыть дашборд. Проверить счётчики задач, просрочку, ближайшие задачи и нагрузку по ответственным.</v>
+        <v>Откройте ссылку и войдите: toniem2@mail.ru / X7mP2vK9qL4bZ1rW. На странице «Дашборд» проверьте карточки со статистикой: всего задач, к выполнению, в работе, просрочено. Ниже проверьте блок ближайших задач и нагрузку по ответственным. Ожидаемый результат: страница показывает статистику использования и текущего состояния задач.</v>
       </c>
     </row>
     <row r="13">
@@ -544,7 +544,7 @@
         <v>http://111.88.245.141/app/admin/analytics</v>
       </c>
       <c r="C13" t="str">
-        <v>Войти и открыть скрытую аналитику. Проверить импорт протоколов, источники задач, completion rate и активность.</v>
+        <v>Откройте ссылку и войдите: toniem2@mail.ru / X7mP2vK9qL4bZ1rW. Это скрытая страница аналитики. Проверьте показатели: загружено протоколов, активные импорты, извлечённые задачи, всего задач, завершённые задачи, источники задач и completion rate. Ожидаемый результат: доступна отдельная аналитика воронки/использования продукта, не вынесенная в основное меню.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>